<commit_message>
[GH243] feat(changesets): GH243 sprint1 — retrait du changeset, réouverture uniforme par le statut
- Objet changeset retiré (types, services, IPC, MCP, vue, graphe, préférence changeTracking) ;
  fichiers changesets/ ignorés, leurs IDs réservés ; type changeset et changeTracking ignorés à la
  lecture du schéma.
- Règle de version unique (versionBump) ; vue Word : statut éditable sur un élément verrouillé,
  bouton « Rouvrir en brouillon » retiré.
- Campagne sans baselineRef ni changeset (paramètres à l'état courant).
- Modifications locales et « Impact à vérifier » dans le panneau Version, Constellation dans le
  panneau Exigences.
- Tests unitaires et e2e GH243, e2e adaptés, SPEC mises à jour.

Refs #243

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/desktop/resources/export-templates/Plan de campagne.xlsx
+++ b/apps/desktop/resources/export-templates/Plan de campagne.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>${project.label} — Plan de campagne</t>
   </si>
@@ -26,12 +26,6 @@
   </si>
   <si>
     <t>${campaign.component}</t>
-  </si>
-  <si>
-    <t>Référence</t>
-  </si>
-  <si>
-    <t>${campaign.baselineRef}</t>
   </si>
   <si>
     <t>Révision</t>
@@ -561,57 +555,49 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="F9" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" s="6">
         <f>COUNTA(A9:A9)</f>

</xml_diff>